<commit_message>
Modifica el nombre de la actividad "Tranvía" para que coincida con la del dataset original.
</commit_message>
<xml_diff>
--- a/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aleja\Documents\Proyectos\concurso-datos-cabildotf-appvivienda\recursos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB72F970-C508-432D-BF61-4E2A6FA17F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E198E79-C84B-4309-94BD-47B57D65C4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Salud" sheetId="1" r:id="rId1"/>
@@ -437,7 +437,7 @@
     <t>Guagua</t>
   </si>
   <si>
-    <t>Tranvía</t>
+    <t>Tranvia</t>
   </si>
 </sst>
 </file>
@@ -447,11 +447,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -559,49 +566,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -847,7 +857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:5" ht="66">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -861,7 +871,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
+    <row r="4" spans="2:5" ht="13.8">
       <c r="B4" s="18" t="s">
         <v>8</v>
       </c>
@@ -875,7 +885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="2:5" ht="13.8">
       <c r="B5" s="19"/>
       <c r="C5" s="4" t="s">
         <v>10</v>
@@ -887,7 +897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="2:5" ht="13.8">
       <c r="B6" s="20"/>
       <c r="C6" s="6" t="s">
         <v>11</v>
@@ -899,7 +909,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
+    <row r="7" spans="2:5" ht="13.8">
       <c r="B7" s="21" t="s">
         <v>12</v>
       </c>
@@ -913,7 +923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:5">
+    <row r="8" spans="2:5" ht="13.8">
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>14</v>
@@ -925,7 +935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:5">
+    <row r="9" spans="2:5" ht="13.8">
       <c r="B9" s="19"/>
       <c r="C9" s="4" t="s">
         <v>15</v>
@@ -937,7 +947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="2:5" ht="13.8">
       <c r="B10" s="19"/>
       <c r="C10" s="4" t="s">
         <v>16</v>
@@ -949,7 +959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5">
+    <row r="11" spans="2:5" ht="13.8">
       <c r="B11" s="19"/>
       <c r="C11" s="8" t="s">
         <v>17</v>
@@ -961,7 +971,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" spans="2:5" ht="13.8">
       <c r="B12" s="19"/>
       <c r="C12" s="9" t="s">
         <v>18</v>
@@ -973,7 +983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:5" ht="13.8">
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
         <v>19</v>
@@ -985,7 +995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="2:5">
+    <row r="14" spans="2:5" ht="13.8">
       <c r="B14" s="19"/>
       <c r="C14" s="9" t="s">
         <v>20</v>
@@ -997,37 +1007,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="2:5" ht="13.8">
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="3:5">
+    <row r="17" spans="3:5" ht="13.8">
       <c r="C17" s="4"/>
     </row>
-    <row r="18" spans="3:5">
+    <row r="18" spans="3:5" ht="13.8">
       <c r="C18" s="4"/>
     </row>
-    <row r="19" spans="3:5">
+    <row r="19" spans="3:5" ht="13.8">
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="3:5">
+    <row r="20" spans="3:5" ht="13.8">
       <c r="C20" s="4"/>
     </row>
-    <row r="21" spans="3:5">
+    <row r="21" spans="3:5" ht="13.8">
       <c r="C21" s="4"/>
     </row>
-    <row r="22" spans="3:5">
+    <row r="22" spans="3:5" ht="13.8">
       <c r="C22" s="4"/>
     </row>
-    <row r="23" spans="3:5">
+    <row r="23" spans="3:5" ht="13.8">
       <c r="C23" s="4"/>
     </row>
-    <row r="24" spans="3:5">
+    <row r="24" spans="3:5" ht="13.8">
       <c r="C24" s="4"/>
     </row>
-    <row r="25" spans="3:5">
+    <row r="25" spans="3:5" ht="13.8">
       <c r="C25" s="4"/>
     </row>
-    <row r="26" spans="3:5">
+    <row r="26" spans="3:5" ht="13.8">
       <c r="C26" s="9"/>
     </row>
     <row r="27" spans="3:5" ht="13.8">
@@ -1126,7 +1136,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:5" ht="66">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1140,7 +1150,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
+    <row r="4" spans="2:5" ht="13.8">
       <c r="B4" s="18" t="s">
         <v>21</v>
       </c>
@@ -1154,7 +1164,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="2:5" ht="13.8">
       <c r="B5" s="19"/>
       <c r="C5" s="4" t="s">
         <v>23</v>
@@ -1166,7 +1176,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="2:5" ht="13.8">
       <c r="B6" s="19"/>
       <c r="C6" s="4" t="s">
         <v>24</v>
@@ -1178,7 +1188,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
+    <row r="7" spans="2:5" ht="13.8">
       <c r="B7" s="19"/>
       <c r="C7" s="4" t="s">
         <v>25</v>
@@ -1190,7 +1200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:5">
+    <row r="8" spans="2:5" ht="13.8">
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>26</v>
@@ -1202,7 +1212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:5">
+    <row r="9" spans="2:5" ht="13.8">
       <c r="B9" s="19"/>
       <c r="C9" s="4" t="s">
         <v>27</v>
@@ -1214,7 +1224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="2:5" ht="13.8">
       <c r="B10" s="19"/>
       <c r="C10" s="4" t="s">
         <v>28</v>
@@ -1226,7 +1236,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:5">
+    <row r="11" spans="2:5" ht="13.8">
       <c r="B11" s="19"/>
       <c r="C11" s="4" t="s">
         <v>29</v>
@@ -1238,7 +1248,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" spans="2:5" ht="13.8">
       <c r="B12" s="19"/>
       <c r="C12" s="4" t="s">
         <v>30</v>
@@ -1250,7 +1260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:5" ht="13.8">
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
         <v>31</v>
@@ -1262,7 +1272,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="2:5">
+    <row r="14" spans="2:5" ht="13.8">
       <c r="B14" s="20"/>
       <c r="C14" s="12" t="s">
         <v>32</v>
@@ -1274,7 +1284,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:5">
+    <row r="15" spans="2:5" ht="13.8">
       <c r="B15" s="18" t="s">
         <v>33</v>
       </c>
@@ -1288,7 +1298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="2:5" ht="13.8">
       <c r="B16" s="19"/>
       <c r="C16" s="4" t="s">
         <v>35</v>
@@ -1300,7 +1310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:5" ht="13.8">
       <c r="B17" s="19"/>
       <c r="C17" s="4" t="s">
         <v>36</v>
@@ -1312,7 +1322,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:5" ht="13.8">
       <c r="B18" s="19"/>
       <c r="C18" s="4" t="s">
         <v>37</v>
@@ -1324,28 +1334,28 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="2:5">
+    <row r="19" spans="2:5" ht="13.8">
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="2:5">
+    <row r="20" spans="2:5" ht="13.8">
       <c r="C20" s="4"/>
     </row>
-    <row r="21" spans="2:5">
+    <row r="21" spans="2:5" ht="13.8">
       <c r="C21" s="4"/>
     </row>
-    <row r="22" spans="2:5">
+    <row r="22" spans="2:5" ht="13.8">
       <c r="C22" s="4"/>
     </row>
-    <row r="23" spans="2:5">
+    <row r="23" spans="2:5" ht="13.8">
       <c r="C23" s="4"/>
     </row>
-    <row r="24" spans="2:5">
+    <row r="24" spans="2:5" ht="13.8">
       <c r="C24" s="4"/>
     </row>
-    <row r="25" spans="2:5">
+    <row r="25" spans="2:5" ht="13.8">
       <c r="C25" s="4"/>
     </row>
-    <row r="26" spans="2:5">
+    <row r="26" spans="2:5" ht="13.8">
       <c r="C26" s="4"/>
     </row>
     <row r="27" spans="2:5" ht="13.8">
@@ -1438,7 +1448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:5" ht="66">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1452,7 +1462,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
+    <row r="4" spans="2:5" ht="13.8">
       <c r="B4" s="23" t="s">
         <v>39</v>
       </c>
@@ -1466,7 +1476,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="2:5" ht="13.8">
       <c r="B5" s="19"/>
       <c r="C5" s="9" t="s">
         <v>41</v>
@@ -1478,7 +1488,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="2:5" ht="13.8">
       <c r="B6" s="19"/>
       <c r="C6" s="9" t="s">
         <v>42</v>
@@ -1490,7 +1500,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
+    <row r="7" spans="2:5" ht="13.8">
       <c r="B7" s="19"/>
       <c r="C7" s="9" t="s">
         <v>43</v>
@@ -1502,7 +1512,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:5">
+    <row r="8" spans="2:5" ht="13.8">
       <c r="B8" s="19"/>
       <c r="C8" s="9" t="s">
         <v>44</v>
@@ -1514,7 +1524,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:5">
+    <row r="9" spans="2:5" ht="13.8">
       <c r="B9" s="19"/>
       <c r="C9" s="9" t="s">
         <v>45</v>
@@ -1526,7 +1536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="2:5" ht="13.8">
       <c r="B10" s="20"/>
       <c r="C10" s="6" t="s">
         <v>46</v>
@@ -1538,7 +1548,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:5">
+    <row r="11" spans="2:5" ht="13.8">
       <c r="B11" s="23" t="s">
         <v>47</v>
       </c>
@@ -1552,7 +1562,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" spans="2:5" ht="13.8">
       <c r="B12" s="19"/>
       <c r="C12" s="9" t="s">
         <v>49</v>
@@ -1564,7 +1574,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:5" ht="13.8">
       <c r="B13" s="19"/>
       <c r="C13" s="9" t="s">
         <v>50</v>
@@ -1576,7 +1586,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="2:5">
+    <row r="14" spans="2:5" ht="13.8">
       <c r="B14" s="19"/>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -1588,7 +1598,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5">
+    <row r="15" spans="2:5" ht="13.8">
       <c r="B15" s="22" t="s">
         <v>52</v>
       </c>
@@ -1602,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="2:5" ht="13.8">
       <c r="B16" s="19"/>
       <c r="C16" s="9" t="s">
         <v>54</v>
@@ -1614,7 +1624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:5" ht="13.8">
       <c r="B17" s="19"/>
       <c r="C17" s="9" t="s">
         <v>55</v>
@@ -1626,7 +1636,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:5" ht="13.8">
       <c r="B18" s="19"/>
       <c r="C18" s="9" t="s">
         <v>56</v>
@@ -1638,7 +1648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="2:5">
+    <row r="19" spans="2:5" ht="13.8">
       <c r="B19" s="19"/>
       <c r="C19" s="9" t="s">
         <v>57</v>
@@ -1650,7 +1660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="2:5">
+    <row r="20" spans="2:5" ht="13.8">
       <c r="B20" s="20"/>
       <c r="C20" s="6" t="s">
         <v>58</v>
@@ -1662,7 +1672,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:5">
+    <row r="21" spans="2:5" ht="13.8">
       <c r="B21" s="23" t="s">
         <v>59</v>
       </c>
@@ -1676,7 +1686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:5">
+    <row r="22" spans="2:5" ht="13.8">
       <c r="B22" s="19"/>
       <c r="C22" s="9" t="s">
         <v>61</v>
@@ -1688,7 +1698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:5">
+    <row r="23" spans="2:5" ht="13.8">
       <c r="B23" s="19"/>
       <c r="C23" s="9" t="s">
         <v>62</v>
@@ -1700,7 +1710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:5">
+    <row r="24" spans="2:5" ht="13.8">
       <c r="B24" s="19"/>
       <c r="C24" s="9" t="s">
         <v>63</v>
@@ -1712,7 +1722,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="2:5">
+    <row r="25" spans="2:5" ht="13.8">
       <c r="B25" s="19"/>
       <c r="C25" s="9" t="s">
         <v>64</v>
@@ -1724,7 +1734,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="2:5">
+    <row r="26" spans="2:5" ht="13.8">
       <c r="B26" s="19"/>
       <c r="C26" s="9" t="s">
         <v>65</v>
@@ -2032,7 +2042,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:5" ht="66">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2046,7 +2056,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
+    <row r="4" spans="2:5" ht="13.8">
       <c r="B4" s="18" t="s">
         <v>89</v>
       </c>
@@ -2060,7 +2070,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="2:5" ht="13.8">
       <c r="B5" s="19"/>
       <c r="C5" s="9" t="s">
         <v>91</v>
@@ -2072,7 +2082,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="2:5" ht="13.8">
       <c r="B6" s="19"/>
       <c r="C6" s="9" t="s">
         <v>92</v>
@@ -2084,7 +2094,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
+    <row r="7" spans="2:5" ht="13.8">
       <c r="B7" s="19"/>
       <c r="C7" s="9" t="s">
         <v>93</v>
@@ -2096,7 +2106,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:5">
+    <row r="8" spans="2:5" ht="13.8">
       <c r="B8" s="19"/>
       <c r="C8" s="9" t="s">
         <v>94</v>
@@ -2108,7 +2118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:5">
+    <row r="9" spans="2:5" ht="13.8">
       <c r="B9" s="19"/>
       <c r="C9" s="9" t="s">
         <v>95</v>
@@ -2120,7 +2130,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="2:5" ht="13.8">
       <c r="B10" s="19"/>
       <c r="C10" s="9" t="s">
         <v>96</v>
@@ -2132,7 +2142,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:5">
+    <row r="11" spans="2:5" ht="13.8">
       <c r="B11" s="19"/>
       <c r="C11" s="9" t="s">
         <v>97</v>
@@ -2144,7 +2154,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" spans="2:5" ht="13.8">
       <c r="B12" s="19"/>
       <c r="C12" s="9" t="s">
         <v>98</v>
@@ -2156,7 +2166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:5" ht="13.8">
       <c r="B13" s="19"/>
       <c r="C13" s="9" t="s">
         <v>99</v>
@@ -2168,7 +2178,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="2:5">
+    <row r="14" spans="2:5" ht="13.8">
       <c r="B14" s="19"/>
       <c r="C14" s="9" t="s">
         <v>100</v>
@@ -2180,7 +2190,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5">
+    <row r="15" spans="2:5" ht="13.8">
       <c r="B15" s="19"/>
       <c r="C15" s="9" t="s">
         <v>101</v>
@@ -2192,7 +2202,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="2:5" ht="13.8">
       <c r="B16" s="21" t="s">
         <v>102</v>
       </c>
@@ -2206,7 +2216,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:5" ht="13.8">
       <c r="B17" s="19"/>
       <c r="C17" s="9" t="s">
         <v>104</v>
@@ -2218,7 +2228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:5" ht="13.8">
       <c r="B18" s="19"/>
       <c r="C18" s="9" t="s">
         <v>105</v>
@@ -2230,7 +2240,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="2:5">
+    <row r="19" spans="2:5" ht="13.8">
       <c r="B19" s="19"/>
       <c r="C19" s="9" t="s">
         <v>106</v>
@@ -2242,7 +2252,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="2:5">
+    <row r="20" spans="2:5" ht="13.8">
       <c r="B20" s="19"/>
       <c r="C20" s="9" t="s">
         <v>107</v>
@@ -2254,7 +2264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:5">
+    <row r="21" spans="2:5" ht="13.8">
       <c r="B21" s="19"/>
       <c r="C21" s="9" t="s">
         <v>108</v>
@@ -2266,7 +2276,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="2:5">
+    <row r="22" spans="2:5" ht="13.8">
       <c r="B22" s="19"/>
       <c r="C22" s="9" t="s">
         <v>109</v>
@@ -2278,7 +2288,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5">
+    <row r="23" spans="2:5" ht="13.8">
       <c r="B23" s="19"/>
       <c r="C23" s="9" t="s">
         <v>110</v>
@@ -2290,7 +2300,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:5">
+    <row r="24" spans="2:5" ht="13.8">
       <c r="B24" s="19"/>
       <c r="C24" s="9" t="s">
         <v>111</v>
@@ -2302,7 +2312,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="2:5">
+    <row r="25" spans="2:5" ht="13.8">
       <c r="B25" s="19"/>
       <c r="C25" s="9" t="s">
         <v>112</v>
@@ -2314,7 +2324,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="2:5">
+    <row r="26" spans="2:5" ht="13.8">
       <c r="B26" s="19"/>
       <c r="C26" s="9" t="s">
         <v>113</v>
@@ -2584,7 +2594,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:5" ht="66">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2598,7 +2608,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
+    <row r="4" spans="2:5" ht="13.8">
       <c r="B4" s="23" t="s">
         <v>135</v>
       </c>
@@ -2612,9 +2622,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="2:5" ht="13.8">
       <c r="B5" s="19"/>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="24" t="s">
         <v>137</v>
       </c>
       <c r="D5" s="17">
@@ -2624,127 +2634,127 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="2:5" ht="13.8">
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
     </row>
-    <row r="7" spans="2:5">
+    <row r="7" spans="2:5" ht="13.8">
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
     </row>
-    <row r="8" spans="2:5">
+    <row r="8" spans="2:5" ht="13.8">
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
     </row>
-    <row r="9" spans="2:5">
+    <row r="9" spans="2:5" ht="13.8">
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="2:5" ht="13.8">
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="2:5">
+    <row r="11" spans="2:5" ht="13.8">
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" spans="2:5" ht="13.8">
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:5" ht="13.8">
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
     </row>
-    <row r="14" spans="2:5">
+    <row r="14" spans="2:5" ht="13.8">
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
     </row>
-    <row r="15" spans="2:5">
+    <row r="15" spans="2:5" ht="13.8">
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="2:5" ht="13.8">
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:5" ht="13.8">
       <c r="B17" s="16"/>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:5" ht="13.8">
       <c r="B18" s="16"/>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
     </row>
-    <row r="19" spans="2:5">
+    <row r="19" spans="2:5" ht="13.8">
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
     </row>
-    <row r="20" spans="2:5">
+    <row r="20" spans="2:5" ht="13.8">
       <c r="B20" s="16"/>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
     </row>
-    <row r="21" spans="2:5">
+    <row r="21" spans="2:5" ht="13.8">
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
     </row>
-    <row r="22" spans="2:5">
+    <row r="22" spans="2:5" ht="13.8">
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
     </row>
-    <row r="23" spans="2:5">
+    <row r="23" spans="2:5" ht="13.8">
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
     </row>
-    <row r="24" spans="2:5">
+    <row r="24" spans="2:5" ht="13.8">
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
     </row>
-    <row r="25" spans="2:5">
+    <row r="25" spans="2:5" ht="13.8">
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
     </row>
-    <row r="26" spans="2:5">
+    <row r="26" spans="2:5" ht="13.8">
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>

</xml_diff>

<commit_message>
Reordena el código y el dataset diccionario_config.json sustituyendo macro_categoria por las pestañas que vamos a utilizar en la app. Modifica app.py para dividir en subpestañas el sidebar con los sliders. Cambia el nombre de mascotas en el excel eliminando el (*).
</commit_message>
<xml_diff>
--- a/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aleja\Documents\Proyectos\concurso-datos-cabildotf-appvivienda\recursos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E198E79-C84B-4309-94BD-47B57D65C4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB594A30-381F-4EC1-8975-A68CBB719F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Salud" sheetId="1" r:id="rId1"/>
@@ -284,9 +284,6 @@
     <t>telefonia</t>
   </si>
   <si>
-    <t>Mascotas (*)</t>
-  </si>
-  <si>
     <t>mascotas</t>
   </si>
   <si>
@@ -438,6 +435,9 @@
   </si>
   <si>
     <t>Tranvia</t>
+  </si>
+  <si>
+    <t>Mascotas</t>
   </si>
 </sst>
 </file>
@@ -597,6 +597,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -609,9 +612,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -872,7 +872,7 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="13.8">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -886,7 +886,7 @@
       </c>
     </row>
     <row r="5" spans="2:5" ht="13.8">
-      <c r="B5" s="19"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
@@ -898,7 +898,7 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="13.8">
-      <c r="B6" s="20"/>
+      <c r="B6" s="21"/>
       <c r="C6" s="6" t="s">
         <v>11</v>
       </c>
@@ -910,7 +910,7 @@
       </c>
     </row>
     <row r="7" spans="2:5" ht="13.8">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -924,7 +924,7 @@
       </c>
     </row>
     <row r="8" spans="2:5" ht="13.8">
-      <c r="B8" s="19"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
@@ -936,7 +936,7 @@
       </c>
     </row>
     <row r="9" spans="2:5" ht="13.8">
-      <c r="B9" s="19"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="4" t="s">
         <v>15</v>
       </c>
@@ -948,7 +948,7 @@
       </c>
     </row>
     <row r="10" spans="2:5" ht="13.8">
-      <c r="B10" s="19"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="4" t="s">
         <v>16</v>
       </c>
@@ -960,7 +960,7 @@
       </c>
     </row>
     <row r="11" spans="2:5" ht="13.8">
-      <c r="B11" s="19"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="8" t="s">
         <v>17</v>
       </c>
@@ -972,7 +972,7 @@
       </c>
     </row>
     <row r="12" spans="2:5" ht="13.8">
-      <c r="B12" s="19"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
         <v>18</v>
       </c>
@@ -984,7 +984,7 @@
       </c>
     </row>
     <row r="13" spans="2:5" ht="13.8">
-      <c r="B13" s="19"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="4" t="s">
         <v>19</v>
       </c>
@@ -996,7 +996,7 @@
       </c>
     </row>
     <row r="14" spans="2:5" ht="13.8">
-      <c r="B14" s="19"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="9" t="s">
         <v>20</v>
       </c>
@@ -1151,7 +1151,7 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="13.8">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -1165,7 +1165,7 @@
       </c>
     </row>
     <row r="5" spans="2:5" ht="13.8">
-      <c r="B5" s="19"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="4" t="s">
         <v>23</v>
       </c>
@@ -1177,7 +1177,7 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="13.8">
-      <c r="B6" s="19"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="4" t="s">
         <v>24</v>
       </c>
@@ -1189,7 +1189,7 @@
       </c>
     </row>
     <row r="7" spans="2:5" ht="13.8">
-      <c r="B7" s="19"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="4" t="s">
         <v>25</v>
       </c>
@@ -1201,7 +1201,7 @@
       </c>
     </row>
     <row r="8" spans="2:5" ht="13.8">
-      <c r="B8" s="19"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="4" t="s">
         <v>26</v>
       </c>
@@ -1213,7 +1213,7 @@
       </c>
     </row>
     <row r="9" spans="2:5" ht="13.8">
-      <c r="B9" s="19"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="4" t="s">
         <v>27</v>
       </c>
@@ -1225,7 +1225,7 @@
       </c>
     </row>
     <row r="10" spans="2:5" ht="13.8">
-      <c r="B10" s="19"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="4" t="s">
         <v>28</v>
       </c>
@@ -1237,7 +1237,7 @@
       </c>
     </row>
     <row r="11" spans="2:5" ht="13.8">
-      <c r="B11" s="19"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="4" t="s">
         <v>29</v>
       </c>
@@ -1249,7 +1249,7 @@
       </c>
     </row>
     <row r="12" spans="2:5" ht="13.8">
-      <c r="B12" s="19"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="4" t="s">
         <v>30</v>
       </c>
@@ -1261,7 +1261,7 @@
       </c>
     </row>
     <row r="13" spans="2:5" ht="13.8">
-      <c r="B13" s="19"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="4" t="s">
         <v>31</v>
       </c>
@@ -1273,7 +1273,7 @@
       </c>
     </row>
     <row r="14" spans="2:5" ht="13.8">
-      <c r="B14" s="20"/>
+      <c r="B14" s="21"/>
       <c r="C14" s="12" t="s">
         <v>32</v>
       </c>
@@ -1285,7 +1285,7 @@
       </c>
     </row>
     <row r="15" spans="2:5" ht="13.8">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -1299,7 +1299,7 @@
       </c>
     </row>
     <row r="16" spans="2:5" ht="13.8">
-      <c r="B16" s="19"/>
+      <c r="B16" s="20"/>
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
@@ -1311,7 +1311,7 @@
       </c>
     </row>
     <row r="17" spans="2:5" ht="13.8">
-      <c r="B17" s="19"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="4" t="s">
         <v>36</v>
       </c>
@@ -1323,7 +1323,7 @@
       </c>
     </row>
     <row r="18" spans="2:5" ht="13.8">
-      <c r="B18" s="19"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="4" t="s">
         <v>37</v>
       </c>
@@ -1463,7 +1463,7 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="13.8">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="9" t="s">
@@ -1477,7 +1477,7 @@
       </c>
     </row>
     <row r="5" spans="2:5" ht="13.8">
-      <c r="B5" s="19"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="9" t="s">
         <v>41</v>
       </c>
@@ -1489,7 +1489,7 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="13.8">
-      <c r="B6" s="19"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="9" t="s">
         <v>42</v>
       </c>
@@ -1501,7 +1501,7 @@
       </c>
     </row>
     <row r="7" spans="2:5" ht="13.8">
-      <c r="B7" s="19"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="9" t="s">
         <v>43</v>
       </c>
@@ -1513,7 +1513,7 @@
       </c>
     </row>
     <row r="8" spans="2:5" ht="13.8">
-      <c r="B8" s="19"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="9" t="s">
         <v>44</v>
       </c>
@@ -1525,7 +1525,7 @@
       </c>
     </row>
     <row r="9" spans="2:5" ht="13.8">
-      <c r="B9" s="19"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="9" t="s">
         <v>45</v>
       </c>
@@ -1537,7 +1537,7 @@
       </c>
     </row>
     <row r="10" spans="2:5" ht="13.8">
-      <c r="B10" s="20"/>
+      <c r="B10" s="21"/>
       <c r="C10" s="6" t="s">
         <v>46</v>
       </c>
@@ -1549,7 +1549,7 @@
       </c>
     </row>
     <row r="11" spans="2:5" ht="13.8">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>47</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -1563,7 +1563,7 @@
       </c>
     </row>
     <row r="12" spans="2:5" ht="13.8">
-      <c r="B12" s="19"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
         <v>49</v>
       </c>
@@ -1575,7 +1575,7 @@
       </c>
     </row>
     <row r="13" spans="2:5" ht="13.8">
-      <c r="B13" s="19"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="9" t="s">
         <v>50</v>
       </c>
@@ -1587,7 +1587,7 @@
       </c>
     </row>
     <row r="14" spans="2:5" ht="13.8">
-      <c r="B14" s="19"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="9" t="s">
         <v>51</v>
       </c>
@@ -1599,7 +1599,7 @@
       </c>
     </row>
     <row r="15" spans="2:5" ht="13.8">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="23" t="s">
         <v>52</v>
       </c>
       <c r="C15" s="13" t="s">
@@ -1613,7 +1613,7 @@
       </c>
     </row>
     <row r="16" spans="2:5" ht="13.8">
-      <c r="B16" s="19"/>
+      <c r="B16" s="20"/>
       <c r="C16" s="9" t="s">
         <v>54</v>
       </c>
@@ -1625,7 +1625,7 @@
       </c>
     </row>
     <row r="17" spans="2:5" ht="13.8">
-      <c r="B17" s="19"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="9" t="s">
         <v>55</v>
       </c>
@@ -1637,7 +1637,7 @@
       </c>
     </row>
     <row r="18" spans="2:5" ht="13.8">
-      <c r="B18" s="19"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="9" t="s">
         <v>56</v>
       </c>
@@ -1649,7 +1649,7 @@
       </c>
     </row>
     <row r="19" spans="2:5" ht="13.8">
-      <c r="B19" s="19"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="9" t="s">
         <v>57</v>
       </c>
@@ -1661,7 +1661,7 @@
       </c>
     </row>
     <row r="20" spans="2:5" ht="13.8">
-      <c r="B20" s="20"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="6" t="s">
         <v>58</v>
       </c>
@@ -1673,7 +1673,7 @@
       </c>
     </row>
     <row r="21" spans="2:5" ht="13.8">
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="24" t="s">
         <v>59</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -1687,7 +1687,7 @@
       </c>
     </row>
     <row r="22" spans="2:5" ht="13.8">
-      <c r="B22" s="19"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="9" t="s">
         <v>61</v>
       </c>
@@ -1699,7 +1699,7 @@
       </c>
     </row>
     <row r="23" spans="2:5" ht="13.8">
-      <c r="B23" s="19"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="9" t="s">
         <v>62</v>
       </c>
@@ -1711,7 +1711,7 @@
       </c>
     </row>
     <row r="24" spans="2:5" ht="13.8">
-      <c r="B24" s="19"/>
+      <c r="B24" s="20"/>
       <c r="C24" s="9" t="s">
         <v>63</v>
       </c>
@@ -1723,7 +1723,7 @@
       </c>
     </row>
     <row r="25" spans="2:5" ht="13.8">
-      <c r="B25" s="19"/>
+      <c r="B25" s="20"/>
       <c r="C25" s="9" t="s">
         <v>64</v>
       </c>
@@ -1735,7 +1735,7 @@
       </c>
     </row>
     <row r="26" spans="2:5" ht="13.8">
-      <c r="B26" s="19"/>
+      <c r="B26" s="20"/>
       <c r="C26" s="9" t="s">
         <v>65</v>
       </c>
@@ -1747,7 +1747,7 @@
       </c>
     </row>
     <row r="27" spans="2:5" ht="13.8">
-      <c r="B27" s="19"/>
+      <c r="B27" s="20"/>
       <c r="C27" s="9" t="s">
         <v>66</v>
       </c>
@@ -1759,7 +1759,7 @@
       </c>
     </row>
     <row r="28" spans="2:5" ht="13.8">
-      <c r="B28" s="19"/>
+      <c r="B28" s="20"/>
       <c r="C28" s="9" t="s">
         <v>67</v>
       </c>
@@ -1771,7 +1771,7 @@
       </c>
     </row>
     <row r="29" spans="2:5" ht="13.8">
-      <c r="B29" s="19"/>
+      <c r="B29" s="20"/>
       <c r="C29" s="9" t="s">
         <v>68</v>
       </c>
@@ -1783,7 +1783,7 @@
       </c>
     </row>
     <row r="30" spans="2:5" ht="13.8">
-      <c r="B30" s="19"/>
+      <c r="B30" s="20"/>
       <c r="C30" s="9" t="s">
         <v>69</v>
       </c>
@@ -1795,7 +1795,7 @@
       </c>
     </row>
     <row r="31" spans="2:5" ht="13.8">
-      <c r="B31" s="19"/>
+      <c r="B31" s="20"/>
       <c r="C31" s="9" t="s">
         <v>70</v>
       </c>
@@ -1807,7 +1807,7 @@
       </c>
     </row>
     <row r="32" spans="2:5" ht="13.8">
-      <c r="B32" s="20"/>
+      <c r="B32" s="21"/>
       <c r="C32" s="6" t="s">
         <v>71</v>
       </c>
@@ -1819,7 +1819,7 @@
       </c>
     </row>
     <row r="33" spans="2:5" ht="13.8">
-      <c r="B33" s="23" t="s">
+      <c r="B33" s="24" t="s">
         <v>72</v>
       </c>
       <c r="C33" s="9" t="s">
@@ -1833,7 +1833,7 @@
       </c>
     </row>
     <row r="34" spans="2:5" ht="13.8">
-      <c r="B34" s="19"/>
+      <c r="B34" s="20"/>
       <c r="C34" s="9" t="s">
         <v>74</v>
       </c>
@@ -1845,7 +1845,7 @@
       </c>
     </row>
     <row r="35" spans="2:5" ht="13.8">
-      <c r="B35" s="19"/>
+      <c r="B35" s="20"/>
       <c r="C35" s="9" t="s">
         <v>75</v>
       </c>
@@ -1857,7 +1857,7 @@
       </c>
     </row>
     <row r="36" spans="2:5" ht="13.8">
-      <c r="B36" s="19"/>
+      <c r="B36" s="20"/>
       <c r="C36" s="9" t="s">
         <v>76</v>
       </c>
@@ -1869,7 +1869,7 @@
       </c>
     </row>
     <row r="37" spans="2:5" ht="13.8">
-      <c r="B37" s="19"/>
+      <c r="B37" s="20"/>
       <c r="C37" s="9" t="s">
         <v>77</v>
       </c>
@@ -1881,7 +1881,7 @@
       </c>
     </row>
     <row r="38" spans="2:5" ht="13.8">
-      <c r="B38" s="19"/>
+      <c r="B38" s="20"/>
       <c r="C38" s="9" t="s">
         <v>78</v>
       </c>
@@ -1893,7 +1893,7 @@
       </c>
     </row>
     <row r="39" spans="2:5" ht="13.8">
-      <c r="B39" s="19"/>
+      <c r="B39" s="20"/>
       <c r="C39" s="9" t="s">
         <v>79</v>
       </c>
@@ -1905,7 +1905,7 @@
       </c>
     </row>
     <row r="40" spans="2:5" ht="13.8">
-      <c r="B40" s="19"/>
+      <c r="B40" s="20"/>
       <c r="C40" s="9" t="s">
         <v>80</v>
       </c>
@@ -1917,7 +1917,7 @@
       </c>
     </row>
     <row r="41" spans="2:5" ht="13.8">
-      <c r="B41" s="19"/>
+      <c r="B41" s="20"/>
       <c r="C41" s="9" t="s">
         <v>81</v>
       </c>
@@ -1929,7 +1929,7 @@
       </c>
     </row>
     <row r="42" spans="2:5" ht="13.8">
-      <c r="B42" s="19"/>
+      <c r="B42" s="20"/>
       <c r="C42" s="9" t="s">
         <v>82</v>
       </c>
@@ -1941,7 +1941,7 @@
       </c>
     </row>
     <row r="43" spans="2:5" ht="13.8">
-      <c r="B43" s="19"/>
+      <c r="B43" s="20"/>
       <c r="C43" s="9" t="s">
         <v>83</v>
       </c>
@@ -1953,7 +1953,7 @@
       </c>
     </row>
     <row r="44" spans="2:5" ht="13.8">
-      <c r="B44" s="19"/>
+      <c r="B44" s="20"/>
       <c r="C44" s="9" t="s">
         <v>84</v>
       </c>
@@ -1965,7 +1965,7 @@
       </c>
     </row>
     <row r="45" spans="2:5" ht="13.8">
-      <c r="B45" s="19"/>
+      <c r="B45" s="20"/>
       <c r="C45" s="9" t="s">
         <v>85</v>
       </c>
@@ -1978,10 +1978,10 @@
     </row>
     <row r="46" spans="2:5" ht="13.8">
       <c r="B46" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="C46" s="15" t="s">
         <v>86</v>
-      </c>
-      <c r="C46" s="15" t="s">
-        <v>87</v>
       </c>
       <c r="D46" s="14">
         <v>6</v>
@@ -1991,9 +1991,9 @@
       </c>
     </row>
     <row r="47" spans="2:5" ht="13.8">
-      <c r="B47" s="19"/>
+      <c r="B47" s="20"/>
       <c r="C47" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D47" s="5">
         <v>10</v>
@@ -2057,11 +2057,11 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="13.8">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>89</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>90</v>
       </c>
       <c r="D4" s="5">
         <v>10</v>
@@ -2071,9 +2071,9 @@
       </c>
     </row>
     <row r="5" spans="2:5" ht="13.8">
-      <c r="B5" s="19"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D5" s="5">
         <v>10</v>
@@ -2083,9 +2083,9 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="13.8">
-      <c r="B6" s="19"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D6" s="5">
         <v>8</v>
@@ -2095,9 +2095,9 @@
       </c>
     </row>
     <row r="7" spans="2:5" ht="13.8">
-      <c r="B7" s="19"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D7" s="5">
         <v>9</v>
@@ -2107,9 +2107,9 @@
       </c>
     </row>
     <row r="8" spans="2:5" ht="13.8">
-      <c r="B8" s="19"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D8" s="5">
         <v>8</v>
@@ -2119,9 +2119,9 @@
       </c>
     </row>
     <row r="9" spans="2:5" ht="13.8">
-      <c r="B9" s="19"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D9" s="5">
         <v>8</v>
@@ -2131,9 +2131,9 @@
       </c>
     </row>
     <row r="10" spans="2:5" ht="13.8">
-      <c r="B10" s="19"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D10" s="5">
         <v>8</v>
@@ -2143,9 +2143,9 @@
       </c>
     </row>
     <row r="11" spans="2:5" ht="13.8">
-      <c r="B11" s="19"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D11" s="5">
         <v>9</v>
@@ -2155,9 +2155,9 @@
       </c>
     </row>
     <row r="12" spans="2:5" ht="13.8">
-      <c r="B12" s="19"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D12" s="5">
         <v>9</v>
@@ -2167,9 +2167,9 @@
       </c>
     </row>
     <row r="13" spans="2:5" ht="13.8">
-      <c r="B13" s="19"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D13" s="5">
         <v>9</v>
@@ -2179,9 +2179,9 @@
       </c>
     </row>
     <row r="14" spans="2:5" ht="13.8">
-      <c r="B14" s="19"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D14" s="5">
         <v>8</v>
@@ -2191,9 +2191,9 @@
       </c>
     </row>
     <row r="15" spans="2:5" ht="13.8">
-      <c r="B15" s="19"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D15" s="5">
         <v>8</v>
@@ -2203,11 +2203,11 @@
       </c>
     </row>
     <row r="16" spans="2:5" ht="13.8">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>102</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>103</v>
       </c>
       <c r="D16" s="14">
         <v>5</v>
@@ -2217,9 +2217,9 @@
       </c>
     </row>
     <row r="17" spans="2:5" ht="13.8">
-      <c r="B17" s="19"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D17" s="5">
         <v>4</v>
@@ -2229,9 +2229,9 @@
       </c>
     </row>
     <row r="18" spans="2:5" ht="13.8">
-      <c r="B18" s="19"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D18" s="5">
         <v>10</v>
@@ -2241,9 +2241,9 @@
       </c>
     </row>
     <row r="19" spans="2:5" ht="13.8">
-      <c r="B19" s="19"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" s="5">
         <v>10</v>
@@ -2253,9 +2253,9 @@
       </c>
     </row>
     <row r="20" spans="2:5" ht="13.8">
-      <c r="B20" s="19"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D20" s="5">
         <v>7</v>
@@ -2265,9 +2265,9 @@
       </c>
     </row>
     <row r="21" spans="2:5" ht="13.8">
-      <c r="B21" s="19"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D21" s="5">
         <v>7</v>
@@ -2277,9 +2277,9 @@
       </c>
     </row>
     <row r="22" spans="2:5" ht="13.8">
-      <c r="B22" s="19"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D22" s="5">
         <v>9</v>
@@ -2289,9 +2289,9 @@
       </c>
     </row>
     <row r="23" spans="2:5" ht="13.8">
-      <c r="B23" s="19"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D23" s="5">
         <v>5</v>
@@ -2301,9 +2301,9 @@
       </c>
     </row>
     <row r="24" spans="2:5" ht="13.8">
-      <c r="B24" s="19"/>
+      <c r="B24" s="20"/>
       <c r="C24" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D24" s="5">
         <v>6</v>
@@ -2313,9 +2313,9 @@
       </c>
     </row>
     <row r="25" spans="2:5" ht="13.8">
-      <c r="B25" s="19"/>
+      <c r="B25" s="20"/>
       <c r="C25" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D25" s="5">
         <v>9</v>
@@ -2325,9 +2325,9 @@
       </c>
     </row>
     <row r="26" spans="2:5" ht="13.8">
-      <c r="B26" s="19"/>
+      <c r="B26" s="20"/>
       <c r="C26" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D26" s="5">
         <v>9</v>
@@ -2337,11 +2337,11 @@
       </c>
     </row>
     <row r="27" spans="2:5" ht="13.8">
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>114</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>115</v>
       </c>
       <c r="D27" s="14">
         <v>8</v>
@@ -2351,9 +2351,9 @@
       </c>
     </row>
     <row r="28" spans="2:5" ht="13.8">
-      <c r="B28" s="19"/>
+      <c r="B28" s="20"/>
       <c r="C28" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D28" s="5">
         <v>9</v>
@@ -2363,9 +2363,9 @@
       </c>
     </row>
     <row r="29" spans="2:5" ht="13.8">
-      <c r="B29" s="19"/>
+      <c r="B29" s="20"/>
       <c r="C29" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D29" s="5">
         <v>10</v>
@@ -2375,9 +2375,9 @@
       </c>
     </row>
     <row r="30" spans="2:5" ht="13.8">
-      <c r="B30" s="19"/>
+      <c r="B30" s="20"/>
       <c r="C30" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D30" s="5">
         <v>9</v>
@@ -2387,9 +2387,9 @@
       </c>
     </row>
     <row r="31" spans="2:5" ht="13.8">
-      <c r="B31" s="19"/>
+      <c r="B31" s="20"/>
       <c r="C31" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D31" s="5">
         <v>9</v>
@@ -2399,9 +2399,9 @@
       </c>
     </row>
     <row r="32" spans="2:5" ht="13.8">
-      <c r="B32" s="19"/>
+      <c r="B32" s="20"/>
       <c r="C32" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D32" s="5">
         <v>9</v>
@@ -2411,9 +2411,9 @@
       </c>
     </row>
     <row r="33" spans="2:5" ht="13.8">
-      <c r="B33" s="19"/>
+      <c r="B33" s="20"/>
       <c r="C33" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D33" s="5">
         <v>10</v>
@@ -2423,9 +2423,9 @@
       </c>
     </row>
     <row r="34" spans="2:5" ht="13.8">
-      <c r="B34" s="19"/>
+      <c r="B34" s="20"/>
       <c r="C34" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D34" s="5">
         <v>7</v>
@@ -2435,9 +2435,9 @@
       </c>
     </row>
     <row r="35" spans="2:5" ht="13.8">
-      <c r="B35" s="19"/>
+      <c r="B35" s="20"/>
       <c r="C35" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D35" s="5">
         <v>8</v>
@@ -2447,9 +2447,9 @@
       </c>
     </row>
     <row r="36" spans="2:5" ht="13.8">
-      <c r="B36" s="20"/>
+      <c r="B36" s="21"/>
       <c r="C36" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D36" s="7">
         <v>8</v>
@@ -2459,11 +2459,11 @@
       </c>
     </row>
     <row r="37" spans="2:5" ht="13.8">
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>125</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>126</v>
       </c>
       <c r="D37" s="5">
         <v>7</v>
@@ -2473,9 +2473,9 @@
       </c>
     </row>
     <row r="38" spans="2:5" ht="13.8">
-      <c r="B38" s="19"/>
+      <c r="B38" s="20"/>
       <c r="C38" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D38" s="5">
         <v>8</v>
@@ -2485,9 +2485,9 @@
       </c>
     </row>
     <row r="39" spans="2:5" ht="13.8">
-      <c r="B39" s="19"/>
+      <c r="B39" s="20"/>
       <c r="C39" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D39" s="5">
         <v>8</v>
@@ -2497,9 +2497,9 @@
       </c>
     </row>
     <row r="40" spans="2:5" ht="13.8">
-      <c r="B40" s="19"/>
+      <c r="B40" s="20"/>
       <c r="C40" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D40" s="5">
         <v>9</v>
@@ -2509,9 +2509,9 @@
       </c>
     </row>
     <row r="41" spans="2:5" ht="13.8">
-      <c r="B41" s="19"/>
+      <c r="B41" s="20"/>
       <c r="C41" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D41" s="5">
         <v>10</v>
@@ -2521,9 +2521,9 @@
       </c>
     </row>
     <row r="42" spans="2:5" ht="13.8">
-      <c r="B42" s="19"/>
+      <c r="B42" s="20"/>
       <c r="C42" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D42" s="5">
         <v>10</v>
@@ -2533,9 +2533,9 @@
       </c>
     </row>
     <row r="43" spans="2:5" ht="13.8">
-      <c r="B43" s="19"/>
+      <c r="B43" s="20"/>
       <c r="C43" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D43" s="5">
         <v>9</v>
@@ -2545,9 +2545,9 @@
       </c>
     </row>
     <row r="44" spans="2:5" ht="13.8">
-      <c r="B44" s="19"/>
+      <c r="B44" s="20"/>
       <c r="C44" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D44" s="5">
         <v>8</v>
@@ -2582,7 +2582,7 @@
   <sheetData>
     <row r="2" spans="2:5" ht="15.75" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
@@ -2609,11 +2609,11 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="13.8">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>135</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>136</v>
       </c>
       <c r="D4" s="17">
         <v>10</v>
@@ -2623,9 +2623,9 @@
       </c>
     </row>
     <row r="5" spans="2:5" ht="13.8">
-      <c r="B5" s="19"/>
-      <c r="C5" s="24" t="s">
-        <v>137</v>
+      <c r="B5" s="20"/>
+      <c r="C5" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="D5" s="17">
         <v>10</v>

</xml_diff>

<commit_message>
Añade una nueva columna al excel con el nombre visible en los checkboxes y las agrupaciones de actividades.
</commit_message>
<xml_diff>
--- a/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aleja\Documents\Proyectos\concurso-datos-cabildotf-appvivienda\recursos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB594A30-381F-4EC1-8975-A68CBB719F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB3C13D5-EE40-4771-9629-B84B67515706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Salud" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="209">
   <si>
     <t>Sliders / Grupos</t>
   </si>
@@ -438,6 +438,219 @@
   </si>
   <si>
     <t>Mascotas</t>
+  </si>
+  <si>
+    <t>Nombre agrupado web</t>
+  </si>
+  <si>
+    <t>Nombre visual que se verá en los checkboxes. Sirve también para las agrupaciones entre actividades redundantes.</t>
+  </si>
+  <si>
+    <t>Farmacias</t>
+  </si>
+  <si>
+    <t>Hospitales</t>
+  </si>
+  <si>
+    <t>Centros de salud</t>
+  </si>
+  <si>
+    <t>Clínicas dentales</t>
+  </si>
+  <si>
+    <t>Guarderías</t>
+  </si>
+  <si>
+    <t>Colegios</t>
+  </si>
+  <si>
+    <t>Institutos</t>
+  </si>
+  <si>
+    <t>Universidades</t>
+  </si>
+  <si>
+    <t>Bibliotecas</t>
+  </si>
+  <si>
+    <t>Museos</t>
+  </si>
+  <si>
+    <t>Centros culturales</t>
+  </si>
+  <si>
+    <t>Tiendas de mascotas</t>
+  </si>
+  <si>
+    <t>Veterinarios</t>
+  </si>
+  <si>
+    <t>Peluquerías</t>
+  </si>
+  <si>
+    <t>Discotecas</t>
+  </si>
+  <si>
+    <t>Cervecerías</t>
+  </si>
+  <si>
+    <t>Salones recreativos</t>
+  </si>
+  <si>
+    <t>Paradas de guagua</t>
+  </si>
+  <si>
+    <t>Paradas de tranvía</t>
+  </si>
+  <si>
+    <t>Heladerías</t>
+  </si>
+  <si>
+    <t>Cafeterías</t>
+  </si>
+  <si>
+    <t>Dulcerías</t>
+  </si>
+  <si>
+    <t>Churrerías</t>
+  </si>
+  <si>
+    <t>Centros formación profesional</t>
+  </si>
+  <si>
+    <t>Centros enseñanza adultos</t>
+  </si>
+  <si>
+    <t>Centros enseñanza idiomas</t>
+  </si>
+  <si>
+    <t>Centros educación especial</t>
+  </si>
+  <si>
+    <t>Academias, música y extraescolares</t>
+  </si>
+  <si>
+    <t>Clínicas de podología</t>
+  </si>
+  <si>
+    <t>Clínicas de psicología</t>
+  </si>
+  <si>
+    <t>Clínicas de logopedia</t>
+  </si>
+  <si>
+    <t>Fisioterapia y rehabilitación</t>
+  </si>
+  <si>
+    <t>Servicios asistenciales</t>
+  </si>
+  <si>
+    <t>Clínicas y especialistas privados</t>
+  </si>
+  <si>
+    <t>Laboratorios clínicos</t>
+  </si>
+  <si>
+    <t>Pizzerías</t>
+  </si>
+  <si>
+    <t>Guachinches y bodegas</t>
+  </si>
+  <si>
+    <t>Tascas y tapeo</t>
+  </si>
+  <si>
+    <t>Restaurantes</t>
+  </si>
+  <si>
+    <t>Hamburgueserías</t>
+  </si>
+  <si>
+    <t>Bares</t>
+  </si>
+  <si>
+    <t>Areperas</t>
+  </si>
+  <si>
+    <t>Creperias</t>
+  </si>
+  <si>
+    <t>Supermercados</t>
+  </si>
+  <si>
+    <t>Mercados tradicionales</t>
+  </si>
+  <si>
+    <t>Kioskos</t>
+  </si>
+  <si>
+    <t>Multitiendas</t>
+  </si>
+  <si>
+    <t>Ópticas</t>
+  </si>
+  <si>
+    <t>Herbolarios</t>
+  </si>
+  <si>
+    <t>Ferreterías</t>
+  </si>
+  <si>
+    <t>Floristerías</t>
+  </si>
+  <si>
+    <t>Hogar, Bricolaje y Decoración</t>
+  </si>
+  <si>
+    <t>Suministros Eléctricos e Iluminación</t>
+  </si>
+  <si>
+    <t>Centros comerciales</t>
+  </si>
+  <si>
+    <t>Artesanía y productos tradicionales</t>
+  </si>
+  <si>
+    <t>Joyerías y relojerías</t>
+  </si>
+  <si>
+    <t>Tiendas de Ropa</t>
+  </si>
+  <si>
+    <t>Zapaterías</t>
+  </si>
+  <si>
+    <t>Mercerías</t>
+  </si>
+  <si>
+    <t>Accesorios y Regalos</t>
+  </si>
+  <si>
+    <t>Venta de artículos deportivos</t>
+  </si>
+  <si>
+    <t>Concesionarios</t>
+  </si>
+  <si>
+    <t>Estudios fotografía</t>
+  </si>
+  <si>
+    <t>Jugeterías</t>
+  </si>
+  <si>
+    <t>Papelerías</t>
+  </si>
+  <si>
+    <t>Locutorios</t>
+  </si>
+  <si>
+    <t>Venta de artículos musicales</t>
+  </si>
+  <si>
+    <t>Tiendas especializadas</t>
+  </si>
+  <si>
+    <t>Informática, Telefonía y Tecnología</t>
   </si>
 </sst>
 </file>
@@ -447,7 +660,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -521,6 +734,21 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -566,7 +794,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -614,6 +842,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,18 +1064,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:E48"/>
+  <dimension ref="B1:F48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="28.6640625" customWidth="1"/>
     <col min="4" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="24.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="15.75" customHeight="1">
+    <row r="1" spans="2:6" ht="15.75" customHeight="1">
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="2:5" ht="15.75" customHeight="1">
+    <row r="2" spans="2:6" ht="15.75" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -856,8 +1089,11 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" ht="66">
+      <c r="F2" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="66">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -870,8 +1106,11 @@
       <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="13.8">
+      <c r="F3" s="25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="13.8">
       <c r="B4" s="19" t="s">
         <v>8</v>
       </c>
@@ -884,8 +1123,11 @@
       <c r="E4" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="13.8">
+      <c r="F4" s="26" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="13.8">
       <c r="B5" s="20"/>
       <c r="C5" s="4" t="s">
         <v>10</v>
@@ -896,8 +1138,11 @@
       <c r="E5" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="13.8">
+      <c r="F5" s="26" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="13.8">
       <c r="B6" s="21"/>
       <c r="C6" s="6" t="s">
         <v>11</v>
@@ -908,8 +1153,11 @@
       <c r="E6" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" ht="13.8">
+      <c r="F6" s="26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="13.8">
       <c r="B7" s="22" t="s">
         <v>12</v>
       </c>
@@ -922,8 +1170,11 @@
       <c r="E7" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" ht="13.8">
+      <c r="F7" s="26" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="13.8">
       <c r="B8" s="20"/>
       <c r="C8" s="4" t="s">
         <v>14</v>
@@ -934,8 +1185,11 @@
       <c r="E8" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" ht="13.8">
+      <c r="F8" s="26" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="13.8">
       <c r="B9" s="20"/>
       <c r="C9" s="4" t="s">
         <v>15</v>
@@ -946,8 +1200,11 @@
       <c r="E9" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" ht="13.8">
+      <c r="F9" s="26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="13.8">
       <c r="B10" s="20"/>
       <c r="C10" s="4" t="s">
         <v>16</v>
@@ -958,8 +1215,11 @@
       <c r="E10" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" ht="13.8">
+      <c r="F10" s="26" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="13.8">
       <c r="B11" s="20"/>
       <c r="C11" s="8" t="s">
         <v>17</v>
@@ -970,8 +1230,11 @@
       <c r="E11" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" ht="13.8">
+      <c r="F11" s="26" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="13.8">
       <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
         <v>18</v>
@@ -982,8 +1245,11 @@
       <c r="E12" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" ht="13.8">
+      <c r="F12" s="26" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="13.8">
       <c r="B13" s="20"/>
       <c r="C13" s="4" t="s">
         <v>19</v>
@@ -994,8 +1260,11 @@
       <c r="E13" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="13.8">
+      <c r="F13" s="26" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="13.8">
       <c r="B14" s="20"/>
       <c r="C14" s="9" t="s">
         <v>20</v>
@@ -1006,8 +1275,11 @@
       <c r="E14" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" ht="13.8">
+      <c r="F14" s="26" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="13.8">
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="3:5" ht="13.8">
@@ -1114,15 +1386,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B2:E44"/>
+  <dimension ref="B2:F44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="25.33203125" customWidth="1"/>
     <col min="4" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="32.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="15.75" customHeight="1">
+    <row r="2" spans="2:6" ht="15.75" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1135,8 +1408,11 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" ht="66">
+      <c r="F2" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="132">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1149,8 +1425,11 @@
       <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="13.8">
+      <c r="F3" s="25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="13.8">
       <c r="B4" s="19" t="s">
         <v>21</v>
       </c>
@@ -1163,8 +1442,11 @@
       <c r="E4" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="13.8">
+      <c r="F4" s="26" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="13.8">
       <c r="B5" s="20"/>
       <c r="C5" s="4" t="s">
         <v>23</v>
@@ -1175,8 +1457,11 @@
       <c r="E5" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="13.8">
+      <c r="F5" s="26" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="13.8">
       <c r="B6" s="20"/>
       <c r="C6" s="4" t="s">
         <v>24</v>
@@ -1187,8 +1472,11 @@
       <c r="E6" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" ht="13.8">
+      <c r="F6" s="26" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="13.8">
       <c r="B7" s="20"/>
       <c r="C7" s="4" t="s">
         <v>25</v>
@@ -1199,8 +1487,11 @@
       <c r="E7" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" ht="13.8">
+      <c r="F7" s="26" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="13.8">
       <c r="B8" s="20"/>
       <c r="C8" s="4" t="s">
         <v>26</v>
@@ -1211,8 +1502,11 @@
       <c r="E8" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" ht="13.8">
+      <c r="F8" s="26" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="13.8">
       <c r="B9" s="20"/>
       <c r="C9" s="4" t="s">
         <v>27</v>
@@ -1223,8 +1517,11 @@
       <c r="E9" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" ht="13.8">
+      <c r="F9" s="26" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="13.8">
       <c r="B10" s="20"/>
       <c r="C10" s="4" t="s">
         <v>28</v>
@@ -1235,8 +1532,11 @@
       <c r="E10" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" ht="13.8">
+      <c r="F10" s="26" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="13.8">
       <c r="B11" s="20"/>
       <c r="C11" s="4" t="s">
         <v>29</v>
@@ -1247,8 +1547,11 @@
       <c r="E11" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" ht="13.8">
+      <c r="F11" s="26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="13.8">
       <c r="B12" s="20"/>
       <c r="C12" s="4" t="s">
         <v>30</v>
@@ -1259,8 +1562,11 @@
       <c r="E12" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" ht="13.8">
+      <c r="F12" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="13.8">
       <c r="B13" s="20"/>
       <c r="C13" s="4" t="s">
         <v>31</v>
@@ -1271,8 +1577,11 @@
       <c r="E13" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="13.8">
+      <c r="F13" s="26" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="13.8">
       <c r="B14" s="21"/>
       <c r="C14" s="12" t="s">
         <v>32</v>
@@ -1283,8 +1592,11 @@
       <c r="E14" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" ht="13.8">
+      <c r="F14" s="26" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="13.8">
       <c r="B15" s="19" t="s">
         <v>33</v>
       </c>
@@ -1297,8 +1609,11 @@
       <c r="E15" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" ht="13.8">
+      <c r="F15" s="26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="13.8">
       <c r="B16" s="20"/>
       <c r="C16" s="4" t="s">
         <v>35</v>
@@ -1309,8 +1624,11 @@
       <c r="E16" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" ht="13.8">
+      <c r="F16" s="26" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="13.8">
       <c r="B17" s="20"/>
       <c r="C17" s="4" t="s">
         <v>36</v>
@@ -1321,8 +1639,11 @@
       <c r="E17" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" ht="13.8">
+      <c r="F17" s="26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="13.8">
       <c r="B18" s="20"/>
       <c r="C18" s="4" t="s">
         <v>37</v>
@@ -1333,47 +1654,50 @@
       <c r="E18" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" ht="13.8">
+      <c r="F18" s="26" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="13.8">
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="2:5" ht="13.8">
+    <row r="20" spans="2:6" ht="13.8">
       <c r="C20" s="4"/>
     </row>
-    <row r="21" spans="2:5" ht="13.8">
+    <row r="21" spans="2:6" ht="13.8">
       <c r="C21" s="4"/>
     </row>
-    <row r="22" spans="2:5" ht="13.8">
+    <row r="22" spans="2:6" ht="13.8">
       <c r="C22" s="4"/>
     </row>
-    <row r="23" spans="2:5" ht="13.8">
+    <row r="23" spans="2:6" ht="13.8">
       <c r="C23" s="4"/>
     </row>
-    <row r="24" spans="2:5" ht="13.8">
+    <row r="24" spans="2:6" ht="13.8">
       <c r="C24" s="4"/>
     </row>
-    <row r="25" spans="2:5" ht="13.8">
+    <row r="25" spans="2:6" ht="13.8">
       <c r="C25" s="4"/>
     </row>
-    <row r="26" spans="2:5" ht="13.8">
+    <row r="26" spans="2:6" ht="13.8">
       <c r="C26" s="4"/>
     </row>
-    <row r="27" spans="2:5" ht="13.8">
+    <row r="27" spans="2:6" ht="13.8">
       <c r="C27" s="4"/>
     </row>
-    <row r="28" spans="2:5" ht="13.8">
+    <row r="28" spans="2:6" ht="13.8">
       <c r="C28" s="4"/>
     </row>
-    <row r="29" spans="2:5" ht="13.8">
+    <row r="29" spans="2:6" ht="13.8">
       <c r="C29" s="4"/>
     </row>
-    <row r="30" spans="2:5" ht="13.8">
+    <row r="30" spans="2:6" ht="13.8">
       <c r="C30" s="4"/>
     </row>
-    <row r="31" spans="2:5" ht="13.8">
+    <row r="31" spans="2:6" ht="13.8">
       <c r="C31" s="4"/>
     </row>
-    <row r="32" spans="2:5" ht="13.8">
+    <row r="32" spans="2:6" ht="13.8">
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="3:3" ht="13.8">
@@ -1426,15 +1750,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B2:E47"/>
+  <dimension ref="B2:F47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="45.77734375" customWidth="1"/>
     <col min="4" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="27.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="15.75" customHeight="1">
+    <row r="2" spans="2:6" ht="15.75" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
@@ -1447,8 +1772,11 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" ht="66">
+      <c r="F2" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="132">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1461,8 +1789,11 @@
       <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="13.8">
+      <c r="F3" s="25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="13.8">
       <c r="B4" s="24" t="s">
         <v>39</v>
       </c>
@@ -1475,8 +1806,11 @@
       <c r="E4" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="13.8">
+      <c r="F4" s="26" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="13.8">
       <c r="B5" s="20"/>
       <c r="C5" s="9" t="s">
         <v>41</v>
@@ -1487,8 +1821,11 @@
       <c r="E5" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="13.8">
+      <c r="F5" s="26" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="13.8">
       <c r="B6" s="20"/>
       <c r="C6" s="9" t="s">
         <v>42</v>
@@ -1499,8 +1836,11 @@
       <c r="E6" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" ht="13.8">
+      <c r="F6" s="26" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="13.8">
       <c r="B7" s="20"/>
       <c r="C7" s="9" t="s">
         <v>43</v>
@@ -1511,8 +1851,11 @@
       <c r="E7" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" ht="13.8">
+      <c r="F7" s="26" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="13.8">
       <c r="B8" s="20"/>
       <c r="C8" s="9" t="s">
         <v>44</v>
@@ -1523,8 +1866,11 @@
       <c r="E8" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" ht="13.8">
+      <c r="F8" s="26" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="13.8">
       <c r="B9" s="20"/>
       <c r="C9" s="9" t="s">
         <v>45</v>
@@ -1535,8 +1881,11 @@
       <c r="E9" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" ht="13.8">
+      <c r="F9" s="26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="13.8">
       <c r="B10" s="21"/>
       <c r="C10" s="6" t="s">
         <v>46</v>
@@ -1547,8 +1896,11 @@
       <c r="E10" s="7">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" ht="13.8">
+      <c r="F10" s="26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="13.8">
       <c r="B11" s="24" t="s">
         <v>47</v>
       </c>
@@ -1561,8 +1913,11 @@
       <c r="E11" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" ht="13.8">
+      <c r="F11" s="26" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="13.8">
       <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
         <v>49</v>
@@ -1573,8 +1928,11 @@
       <c r="E12" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" ht="13.8">
+      <c r="F12" s="26" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="13.8">
       <c r="B13" s="20"/>
       <c r="C13" s="9" t="s">
         <v>50</v>
@@ -1585,8 +1943,11 @@
       <c r="E13" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="13.8">
+      <c r="F13" s="26" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="13.8">
       <c r="B14" s="20"/>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -1597,8 +1958,11 @@
       <c r="E14" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" ht="13.8">
+      <c r="F14" s="26" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="13.8">
       <c r="B15" s="23" t="s">
         <v>52</v>
       </c>
@@ -1611,8 +1975,11 @@
       <c r="E15" s="14">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" ht="13.8">
+      <c r="F15" s="26" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="13.8">
       <c r="B16" s="20"/>
       <c r="C16" s="9" t="s">
         <v>54</v>
@@ -1623,8 +1990,11 @@
       <c r="E16" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" ht="13.8">
+      <c r="F16" s="26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="13.8">
       <c r="B17" s="20"/>
       <c r="C17" s="9" t="s">
         <v>55</v>
@@ -1635,8 +2005,11 @@
       <c r="E17" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" ht="13.8">
+      <c r="F17" s="26" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="13.8">
       <c r="B18" s="20"/>
       <c r="C18" s="9" t="s">
         <v>56</v>
@@ -1647,8 +2020,11 @@
       <c r="E18" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" ht="13.8">
+      <c r="F18" s="26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="13.8">
       <c r="B19" s="20"/>
       <c r="C19" s="9" t="s">
         <v>57</v>
@@ -1659,8 +2035,11 @@
       <c r="E19" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" ht="13.8">
+      <c r="F19" s="26" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="13.8">
       <c r="B20" s="21"/>
       <c r="C20" s="6" t="s">
         <v>58</v>
@@ -1671,8 +2050,11 @@
       <c r="E20" s="7">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" ht="13.8">
+      <c r="F20" s="26" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="13.8">
       <c r="B21" s="24" t="s">
         <v>59</v>
       </c>
@@ -1685,8 +2067,11 @@
       <c r="E21" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" ht="13.8">
+      <c r="F21" s="26" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="13.8">
       <c r="B22" s="20"/>
       <c r="C22" s="9" t="s">
         <v>61</v>
@@ -1697,8 +2082,11 @@
       <c r="E22" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" ht="13.8">
+      <c r="F22" s="26" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="13.8">
       <c r="B23" s="20"/>
       <c r="C23" s="9" t="s">
         <v>62</v>
@@ -1709,8 +2097,11 @@
       <c r="E23" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" ht="13.8">
+      <c r="F23" s="26" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="13.8">
       <c r="B24" s="20"/>
       <c r="C24" s="9" t="s">
         <v>63</v>
@@ -1721,8 +2112,11 @@
       <c r="E24" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" ht="13.8">
+      <c r="F24" s="26" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="13.8">
       <c r="B25" s="20"/>
       <c r="C25" s="9" t="s">
         <v>64</v>
@@ -1733,8 +2127,11 @@
       <c r="E25" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" ht="13.8">
+      <c r="F25" s="26" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="13.8">
       <c r="B26" s="20"/>
       <c r="C26" s="9" t="s">
         <v>65</v>
@@ -1745,8 +2142,11 @@
       <c r="E26" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" ht="13.8">
+      <c r="F26" s="26" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="13.8">
       <c r="B27" s="20"/>
       <c r="C27" s="9" t="s">
         <v>66</v>
@@ -1757,8 +2157,11 @@
       <c r="E27" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" ht="13.8">
+      <c r="F27" s="26" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="13.8">
       <c r="B28" s="20"/>
       <c r="C28" s="9" t="s">
         <v>67</v>
@@ -1769,8 +2172,11 @@
       <c r="E28" s="5">
         <v>4</v>
       </c>
-    </row>
-    <row r="29" spans="2:5" ht="13.8">
+      <c r="F28" s="26" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="13.8">
       <c r="B29" s="20"/>
       <c r="C29" s="9" t="s">
         <v>68</v>
@@ -1781,8 +2187,11 @@
       <c r="E29" s="5">
         <v>4</v>
       </c>
-    </row>
-    <row r="30" spans="2:5" ht="13.8">
+      <c r="F29" s="26" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="13.8">
       <c r="B30" s="20"/>
       <c r="C30" s="9" t="s">
         <v>69</v>
@@ -1793,8 +2202,11 @@
       <c r="E30" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="31" spans="2:5" ht="13.8">
+      <c r="F30" s="26" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" ht="13.8">
       <c r="B31" s="20"/>
       <c r="C31" s="9" t="s">
         <v>70</v>
@@ -1805,8 +2217,11 @@
       <c r="E31" s="5">
         <v>4</v>
       </c>
-    </row>
-    <row r="32" spans="2:5" ht="13.8">
+      <c r="F31" s="26" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="13.8">
       <c r="B32" s="21"/>
       <c r="C32" s="6" t="s">
         <v>71</v>
@@ -1817,8 +2232,11 @@
       <c r="E32" s="7">
         <v>2</v>
       </c>
-    </row>
-    <row r="33" spans="2:5" ht="13.8">
+      <c r="F32" s="26" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" ht="13.8">
       <c r="B33" s="24" t="s">
         <v>72</v>
       </c>
@@ -1831,8 +2249,11 @@
       <c r="E33" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="2:5" ht="13.8">
+      <c r="F33" s="26" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="13.8">
       <c r="B34" s="20"/>
       <c r="C34" s="9" t="s">
         <v>74</v>
@@ -1843,8 +2264,11 @@
       <c r="E34" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="2:5" ht="13.8">
+      <c r="F34" s="26" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="13.8">
       <c r="B35" s="20"/>
       <c r="C35" s="9" t="s">
         <v>75</v>
@@ -1855,8 +2279,11 @@
       <c r="E35" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="36" spans="2:5" ht="13.8">
+      <c r="F35" s="26" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="13.8">
       <c r="B36" s="20"/>
       <c r="C36" s="9" t="s">
         <v>76</v>
@@ -1867,8 +2294,11 @@
       <c r="E36" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="37" spans="2:5" ht="13.8">
+      <c r="F36" s="26" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="13.8">
       <c r="B37" s="20"/>
       <c r="C37" s="9" t="s">
         <v>77</v>
@@ -1879,8 +2309,11 @@
       <c r="E37" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="38" spans="2:5" ht="13.8">
+      <c r="F37" s="26" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" ht="13.8">
       <c r="B38" s="20"/>
       <c r="C38" s="9" t="s">
         <v>78</v>
@@ -1891,8 +2324,11 @@
       <c r="E38" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="39" spans="2:5" ht="13.8">
+      <c r="F38" s="26" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" ht="13.8">
       <c r="B39" s="20"/>
       <c r="C39" s="9" t="s">
         <v>79</v>
@@ -1903,8 +2339,11 @@
       <c r="E39" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="2:5" ht="13.8">
+      <c r="F39" s="26" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" ht="13.8">
       <c r="B40" s="20"/>
       <c r="C40" s="9" t="s">
         <v>80</v>
@@ -1915,8 +2354,11 @@
       <c r="E40" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="2:5" ht="13.8">
+      <c r="F40" s="26" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" ht="13.8">
       <c r="B41" s="20"/>
       <c r="C41" s="9" t="s">
         <v>81</v>
@@ -1927,8 +2369,11 @@
       <c r="E41" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="42" spans="2:5" ht="13.8">
+      <c r="F41" s="26" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" ht="13.8">
       <c r="B42" s="20"/>
       <c r="C42" s="9" t="s">
         <v>82</v>
@@ -1939,8 +2384,11 @@
       <c r="E42" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="43" spans="2:5" ht="13.8">
+      <c r="F42" s="26" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" ht="13.8">
       <c r="B43" s="20"/>
       <c r="C43" s="9" t="s">
         <v>83</v>
@@ -1951,8 +2399,11 @@
       <c r="E43" s="5">
         <v>4</v>
       </c>
-    </row>
-    <row r="44" spans="2:5" ht="13.8">
+      <c r="F43" s="26" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" ht="13.8">
       <c r="B44" s="20"/>
       <c r="C44" s="9" t="s">
         <v>84</v>
@@ -1963,8 +2414,11 @@
       <c r="E44" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="45" spans="2:5" ht="13.8">
+      <c r="F44" s="26" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" ht="13.8">
       <c r="B45" s="20"/>
       <c r="C45" s="9" t="s">
         <v>85</v>
@@ -1975,8 +2429,11 @@
       <c r="E45" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="46" spans="2:5" ht="13.8">
+      <c r="F45" s="26" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" ht="13.8">
       <c r="B46" s="22" t="s">
         <v>137</v>
       </c>
@@ -1989,8 +2446,11 @@
       <c r="E46" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="47" spans="2:5" ht="13.8">
+      <c r="F46" s="26" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" ht="13.8">
       <c r="B47" s="20"/>
       <c r="C47" s="9" t="s">
         <v>87</v>
@@ -2000,6 +2460,9 @@
       </c>
       <c r="E47" s="5">
         <v>2</v>
+      </c>
+      <c r="F47" s="26" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -2020,15 +2483,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B2:E44"/>
+  <dimension ref="B2:F44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="25.33203125" customWidth="1"/>
     <col min="4" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="15.75" customHeight="1">
+    <row r="2" spans="2:6" ht="15.75" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2041,8 +2505,11 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" ht="66">
+      <c r="F2" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="132">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2055,8 +2522,11 @@
       <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="13.8">
+      <c r="F3" s="25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="13.8">
       <c r="B4" s="19" t="s">
         <v>88</v>
       </c>
@@ -2069,8 +2539,11 @@
       <c r="E4" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="13.8">
+      <c r="F4" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="13.8">
       <c r="B5" s="20"/>
       <c r="C5" s="9" t="s">
         <v>90</v>
@@ -2081,8 +2554,11 @@
       <c r="E5" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="13.8">
+      <c r="F5" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="13.8">
       <c r="B6" s="20"/>
       <c r="C6" s="9" t="s">
         <v>91</v>
@@ -2093,8 +2569,11 @@
       <c r="E6" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" ht="13.8">
+      <c r="F6" s="26" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="13.8">
       <c r="B7" s="20"/>
       <c r="C7" s="9" t="s">
         <v>92</v>
@@ -2105,8 +2584,11 @@
       <c r="E7" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" ht="13.8">
+      <c r="F7" s="26" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="13.8">
       <c r="B8" s="20"/>
       <c r="C8" s="9" t="s">
         <v>93</v>
@@ -2117,8 +2599,11 @@
       <c r="E8" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" ht="13.8">
+      <c r="F8" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="13.8">
       <c r="B9" s="20"/>
       <c r="C9" s="9" t="s">
         <v>94</v>
@@ -2129,8 +2614,11 @@
       <c r="E9" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" ht="13.8">
+      <c r="F9" s="26" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="13.8">
       <c r="B10" s="20"/>
       <c r="C10" s="9" t="s">
         <v>95</v>
@@ -2141,8 +2629,11 @@
       <c r="E10" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" ht="13.8">
+      <c r="F10" s="26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="13.8">
       <c r="B11" s="20"/>
       <c r="C11" s="9" t="s">
         <v>96</v>
@@ -2153,8 +2644,11 @@
       <c r="E11" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" ht="13.8">
+      <c r="F11" s="26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="13.8">
       <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
         <v>97</v>
@@ -2165,8 +2659,11 @@
       <c r="E12" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" ht="13.8">
+      <c r="F12" s="26" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="13.8">
       <c r="B13" s="20"/>
       <c r="C13" s="9" t="s">
         <v>98</v>
@@ -2177,8 +2674,11 @@
       <c r="E13" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="13.8">
+      <c r="F13" s="26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="13.8">
       <c r="B14" s="20"/>
       <c r="C14" s="9" t="s">
         <v>99</v>
@@ -2189,8 +2689,11 @@
       <c r="E14" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" ht="13.8">
+      <c r="F14" s="26" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="13.8">
       <c r="B15" s="20"/>
       <c r="C15" s="9" t="s">
         <v>100</v>
@@ -2201,8 +2704,11 @@
       <c r="E15" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" ht="13.8">
+      <c r="F15" s="26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="13.8">
       <c r="B16" s="22" t="s">
         <v>101</v>
       </c>
@@ -2215,8 +2721,11 @@
       <c r="E16" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" ht="13.8">
+      <c r="F16" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="13.8">
       <c r="B17" s="20"/>
       <c r="C17" s="9" t="s">
         <v>103</v>
@@ -2227,8 +2736,11 @@
       <c r="E17" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" ht="13.8">
+      <c r="F17" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="13.8">
       <c r="B18" s="20"/>
       <c r="C18" s="9" t="s">
         <v>104</v>
@@ -2239,8 +2751,11 @@
       <c r="E18" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" ht="13.8">
+      <c r="F18" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="13.8">
       <c r="B19" s="20"/>
       <c r="C19" s="9" t="s">
         <v>105</v>
@@ -2251,8 +2766,11 @@
       <c r="E19" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" ht="13.8">
+      <c r="F19" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="13.8">
       <c r="B20" s="20"/>
       <c r="C20" s="9" t="s">
         <v>106</v>
@@ -2263,8 +2781,11 @@
       <c r="E20" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" ht="13.8">
+      <c r="F20" s="26" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="13.8">
       <c r="B21" s="20"/>
       <c r="C21" s="9" t="s">
         <v>107</v>
@@ -2275,8 +2796,11 @@
       <c r="E21" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" ht="13.8">
+      <c r="F21" s="26" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="13.8">
       <c r="B22" s="20"/>
       <c r="C22" s="9" t="s">
         <v>108</v>
@@ -2287,8 +2811,11 @@
       <c r="E22" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" ht="13.8">
+      <c r="F22" s="26" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="13.8">
       <c r="B23" s="20"/>
       <c r="C23" s="9" t="s">
         <v>109</v>
@@ -2299,8 +2826,11 @@
       <c r="E23" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" ht="13.8">
+      <c r="F23" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="13.8">
       <c r="B24" s="20"/>
       <c r="C24" s="9" t="s">
         <v>110</v>
@@ -2311,8 +2841,11 @@
       <c r="E24" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" ht="13.8">
+      <c r="F24" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="13.8">
       <c r="B25" s="20"/>
       <c r="C25" s="9" t="s">
         <v>111</v>
@@ -2323,8 +2856,11 @@
       <c r="E25" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" ht="13.8">
+      <c r="F25" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="13.8">
       <c r="B26" s="20"/>
       <c r="C26" s="9" t="s">
         <v>112</v>
@@ -2335,8 +2871,11 @@
       <c r="E26" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" ht="13.8">
+      <c r="F26" s="26" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="13.8">
       <c r="B27" s="22" t="s">
         <v>113</v>
       </c>
@@ -2349,8 +2888,11 @@
       <c r="E27" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" ht="13.8">
+      <c r="F27" s="26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="13.8">
       <c r="B28" s="20"/>
       <c r="C28" s="9" t="s">
         <v>115</v>
@@ -2361,8 +2903,11 @@
       <c r="E28" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="29" spans="2:5" ht="13.8">
+      <c r="F28" s="26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="13.8">
       <c r="B29" s="20"/>
       <c r="C29" s="9" t="s">
         <v>116</v>
@@ -2373,8 +2918,11 @@
       <c r="E29" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="2:5" ht="13.8">
+      <c r="F29" s="26" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="13.8">
       <c r="B30" s="20"/>
       <c r="C30" s="9" t="s">
         <v>117</v>
@@ -2385,8 +2933,11 @@
       <c r="E30" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="31" spans="2:5" ht="13.8">
+      <c r="F30" s="26" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" ht="13.8">
       <c r="B31" s="20"/>
       <c r="C31" s="9" t="s">
         <v>118</v>
@@ -2397,8 +2948,11 @@
       <c r="E31" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="32" spans="2:5" ht="13.8">
+      <c r="F31" s="26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="13.8">
       <c r="B32" s="20"/>
       <c r="C32" s="9" t="s">
         <v>119</v>
@@ -2409,8 +2963,11 @@
       <c r="E32" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="33" spans="2:5" ht="13.8">
+      <c r="F32" s="26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" ht="13.8">
       <c r="B33" s="20"/>
       <c r="C33" s="9" t="s">
         <v>120</v>
@@ -2421,8 +2978,11 @@
       <c r="E33" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="34" spans="2:5" ht="13.8">
+      <c r="F33" s="26" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="13.8">
       <c r="B34" s="20"/>
       <c r="C34" s="9" t="s">
         <v>121</v>
@@ -2433,8 +2993,11 @@
       <c r="E34" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="2:5" ht="13.8">
+      <c r="F34" s="26" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="13.8">
       <c r="B35" s="20"/>
       <c r="C35" s="9" t="s">
         <v>122</v>
@@ -2445,8 +3008,11 @@
       <c r="E35" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="36" spans="2:5" ht="13.8">
+      <c r="F35" s="26" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="13.8">
       <c r="B36" s="21"/>
       <c r="C36" s="6" t="s">
         <v>123</v>
@@ -2457,8 +3023,11 @@
       <c r="E36" s="7">
         <v>2</v>
       </c>
-    </row>
-    <row r="37" spans="2:5" ht="13.8">
+      <c r="F36" s="26" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="13.8">
       <c r="B37" s="19" t="s">
         <v>124</v>
       </c>
@@ -2471,8 +3040,11 @@
       <c r="E37" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="2:5" ht="13.8">
+      <c r="F37" s="26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" ht="13.8">
       <c r="B38" s="20"/>
       <c r="C38" s="9" t="s">
         <v>126</v>
@@ -2483,8 +3055,11 @@
       <c r="E38" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="39" spans="2:5" ht="13.8">
+      <c r="F38" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" ht="13.8">
       <c r="B39" s="20"/>
       <c r="C39" s="9" t="s">
         <v>127</v>
@@ -2495,8 +3070,11 @@
       <c r="E39" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="40" spans="2:5" ht="13.8">
+      <c r="F39" s="26" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" ht="13.8">
       <c r="B40" s="20"/>
       <c r="C40" s="9" t="s">
         <v>128</v>
@@ -2507,8 +3085,11 @@
       <c r="E40" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="2:5" ht="13.8">
+      <c r="F40" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" ht="13.8">
       <c r="B41" s="20"/>
       <c r="C41" s="9" t="s">
         <v>129</v>
@@ -2519,8 +3100,11 @@
       <c r="E41" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="42" spans="2:5" ht="13.8">
+      <c r="F41" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" ht="13.8">
       <c r="B42" s="20"/>
       <c r="C42" s="9" t="s">
         <v>130</v>
@@ -2531,8 +3115,11 @@
       <c r="E42" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="43" spans="2:5" ht="13.8">
+      <c r="F42" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" ht="13.8">
       <c r="B43" s="20"/>
       <c r="C43" s="9" t="s">
         <v>131</v>
@@ -2543,8 +3130,11 @@
       <c r="E43" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="44" spans="2:5" ht="13.8">
+      <c r="F43" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" ht="13.8">
       <c r="B44" s="20"/>
       <c r="C44" s="9" t="s">
         <v>132</v>
@@ -2554,6 +3144,9 @@
       </c>
       <c r="E44" s="5">
         <v>2</v>
+      </c>
+      <c r="F44" s="26" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2572,15 +3165,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B2:E44"/>
+  <dimension ref="B2:F44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="18.21875" customWidth="1"/>
     <col min="4" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="15.75" customHeight="1">
+    <row r="2" spans="2:6" ht="15.75" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>133</v>
       </c>
@@ -2593,8 +3187,11 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" ht="66">
+      <c r="F2" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="132">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2607,8 +3204,11 @@
       <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="13.8">
+      <c r="F3" s="25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="13.8">
       <c r="B4" s="24" t="s">
         <v>134</v>
       </c>
@@ -2621,8 +3221,11 @@
       <c r="E4" s="17">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="13.8">
+      <c r="F4" s="26" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="13.8">
       <c r="B5" s="20"/>
       <c r="C5" s="18" t="s">
         <v>136</v>
@@ -2633,68 +3236,71 @@
       <c r="E5" s="17">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="13.8">
+      <c r="F5" s="26" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="13.8">
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
     </row>
-    <row r="7" spans="2:5" ht="13.8">
+    <row r="7" spans="2:6" ht="13.8">
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
     </row>
-    <row r="8" spans="2:5" ht="13.8">
+    <row r="8" spans="2:6" ht="13.8">
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
     </row>
-    <row r="9" spans="2:5" ht="13.8">
+    <row r="9" spans="2:6" ht="13.8">
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
     </row>
-    <row r="10" spans="2:5" ht="13.8">
+    <row r="10" spans="2:6" ht="13.8">
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="2:5" ht="13.8">
+    <row r="11" spans="2:6" ht="13.8">
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
     </row>
-    <row r="12" spans="2:5" ht="13.8">
+    <row r="12" spans="2:6" ht="13.8">
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
     </row>
-    <row r="13" spans="2:5" ht="13.8">
+    <row r="13" spans="2:6" ht="13.8">
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
     </row>
-    <row r="14" spans="2:5" ht="13.8">
+    <row r="14" spans="2:6" ht="13.8">
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
     </row>
-    <row r="15" spans="2:5" ht="13.8">
+    <row r="15" spans="2:6" ht="13.8">
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
     </row>
-    <row r="16" spans="2:5" ht="13.8">
+    <row r="16" spans="2:6" ht="13.8">
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>

</xml_diff>

<commit_message>
Cambia el nombre del dataset de equipamientos a naturaleza y limpia el dataset
</commit_message>
<xml_diff>
--- a/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -9,6 +9,7 @@
     <sheet state="visible" name="Restauración" sheetId="4" r:id="rId8"/>
     <sheet state="visible" name="Movilidad" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="Deporte y Ocio" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="Naturaleza" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -16,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="230">
   <si>
     <t>Sliders / Grupos</t>
   </si>
@@ -688,6 +689,24 @@
   </si>
   <si>
     <t>parque deporte urbano</t>
+  </si>
+  <si>
+    <t>Ocio y picnic</t>
+  </si>
+  <si>
+    <t>Area recreativa</t>
+  </si>
+  <si>
+    <t>Areas recreativas</t>
+  </si>
+  <si>
+    <t>Paisaje y vistas</t>
+  </si>
+  <si>
+    <t>Mirador</t>
+  </si>
+  <si>
+    <t>Miradores</t>
   </si>
 </sst>
 </file>
@@ -911,6 +930,10 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -9579,4 +9602,1286 @@
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="12.63"/>
+    <col customWidth="1" min="2" max="2" width="23.75"/>
+    <col customWidth="1" min="3" max="3" width="27.75"/>
+    <col customWidth="1" min="4" max="5" width="23.88"/>
+    <col customWidth="1" min="6" max="6" width="24.88"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="B2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="B4" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" s="25">
+        <v>10.0</v>
+      </c>
+      <c r="E4" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="B5" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="D5" s="27">
+        <v>8.0</v>
+      </c>
+      <c r="E5" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="B9" s="27"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="24"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="B43" s="24"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1"/>
+    <row r="46" ht="15.75" customHeight="1"/>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="51" ht="15.75" customHeight="1"/>
+    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
+    <row r="101" ht="15.75" customHeight="1"/>
+    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1"/>
+    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1"/>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="110" ht="15.75" customHeight="1"/>
+    <row r="111" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1"/>
+    <row r="113" ht="15.75" customHeight="1"/>
+    <row r="114" ht="15.75" customHeight="1"/>
+    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="117" ht="15.75" customHeight="1"/>
+    <row r="118" ht="15.75" customHeight="1"/>
+    <row r="119" ht="15.75" customHeight="1"/>
+    <row r="120" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1"/>
+    <row r="122" ht="15.75" customHeight="1"/>
+    <row r="123" ht="15.75" customHeight="1"/>
+    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="125" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1"/>
+    <row r="127" ht="15.75" customHeight="1"/>
+    <row r="128" ht="15.75" customHeight="1"/>
+    <row r="129" ht="15.75" customHeight="1"/>
+    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="131" ht="15.75" customHeight="1"/>
+    <row r="132" ht="15.75" customHeight="1"/>
+    <row r="133" ht="15.75" customHeight="1"/>
+    <row r="134" ht="15.75" customHeight="1"/>
+    <row r="135" ht="15.75" customHeight="1"/>
+    <row r="136" ht="15.75" customHeight="1"/>
+    <row r="137" ht="15.75" customHeight="1"/>
+    <row r="138" ht="15.75" customHeight="1"/>
+    <row r="139" ht="15.75" customHeight="1"/>
+    <row r="140" ht="15.75" customHeight="1"/>
+    <row r="141" ht="15.75" customHeight="1"/>
+    <row r="142" ht="15.75" customHeight="1"/>
+    <row r="143" ht="15.75" customHeight="1"/>
+    <row r="144" ht="15.75" customHeight="1"/>
+    <row r="145" ht="15.75" customHeight="1"/>
+    <row r="146" ht="15.75" customHeight="1"/>
+    <row r="147" ht="15.75" customHeight="1"/>
+    <row r="148" ht="15.75" customHeight="1"/>
+    <row r="149" ht="15.75" customHeight="1"/>
+    <row r="150" ht="15.75" customHeight="1"/>
+    <row r="151" ht="15.75" customHeight="1"/>
+    <row r="152" ht="15.75" customHeight="1"/>
+    <row r="153" ht="15.75" customHeight="1"/>
+    <row r="154" ht="15.75" customHeight="1"/>
+    <row r="155" ht="15.75" customHeight="1"/>
+    <row r="156" ht="15.75" customHeight="1"/>
+    <row r="157" ht="15.75" customHeight="1"/>
+    <row r="158" ht="15.75" customHeight="1"/>
+    <row r="159" ht="15.75" customHeight="1"/>
+    <row r="160" ht="15.75" customHeight="1"/>
+    <row r="161" ht="15.75" customHeight="1"/>
+    <row r="162" ht="15.75" customHeight="1"/>
+    <row r="163" ht="15.75" customHeight="1"/>
+    <row r="164" ht="15.75" customHeight="1"/>
+    <row r="165" ht="15.75" customHeight="1"/>
+    <row r="166" ht="15.75" customHeight="1"/>
+    <row r="167" ht="15.75" customHeight="1"/>
+    <row r="168" ht="15.75" customHeight="1"/>
+    <row r="169" ht="15.75" customHeight="1"/>
+    <row r="170" ht="15.75" customHeight="1"/>
+    <row r="171" ht="15.75" customHeight="1"/>
+    <row r="172" ht="15.75" customHeight="1"/>
+    <row r="173" ht="15.75" customHeight="1"/>
+    <row r="174" ht="15.75" customHeight="1"/>
+    <row r="175" ht="15.75" customHeight="1"/>
+    <row r="176" ht="15.75" customHeight="1"/>
+    <row r="177" ht="15.75" customHeight="1"/>
+    <row r="178" ht="15.75" customHeight="1"/>
+    <row r="179" ht="15.75" customHeight="1"/>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
+  </sheetData>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Incluye mas actividades en el dataset de naturaleza y añade los mapas visuales para los datasets de centros deportivos y ocio y naturaleza.
</commit_message>
<xml_diff>
--- a/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="242">
   <si>
     <t>Sliders / Grupos</t>
   </si>
@@ -700,6 +700,18 @@
     <t>Areas recreativas</t>
   </si>
   <si>
+    <t>Area de descanso</t>
+  </si>
+  <si>
+    <t>Educacion ambiental</t>
+  </si>
+  <si>
+    <t>Aula en la naturaleza</t>
+  </si>
+  <si>
+    <t>Aulas en la naturaleza</t>
+  </si>
+  <si>
     <t>Paisaje y vistas</t>
   </si>
   <si>
@@ -707,6 +719,30 @@
   </si>
   <si>
     <t>Miradores</t>
+  </si>
+  <si>
+    <t>Centro de visitantes</t>
+  </si>
+  <si>
+    <t>Centros de visitantes</t>
+  </si>
+  <si>
+    <t>Camping</t>
+  </si>
+  <si>
+    <t>Zona de acampada (caravanas)</t>
+  </si>
+  <si>
+    <t>Zonas para acampar</t>
+  </si>
+  <si>
+    <t>Zona de acampada (casetas)</t>
+  </si>
+  <si>
+    <t>Campamento</t>
+  </si>
+  <si>
+    <t>Zona vivac</t>
   </si>
 </sst>
 </file>
@@ -9672,11 +9708,8 @@
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="B5" s="27" t="s">
+      <c r="C5" s="27" t="s">
         <v>227</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>228</v>
       </c>
       <c r="D5" s="27">
         <v>8.0</v>
@@ -9685,50 +9718,115 @@
         <v>1.0</v>
       </c>
       <c r="F5" s="29" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="B6" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="C6" s="27" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
+      <c r="D6" s="27">
+        <v>5.0</v>
+      </c>
+      <c r="E6" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
+      <c r="B7" s="27" t="s">
+        <v>231</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="27">
+        <v>8.0</v>
+      </c>
+      <c r="E7" s="27">
+        <v>2.0</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
+      <c r="C8" s="27" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" s="27">
+        <v>5.0</v>
+      </c>
+      <c r="E8" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="B9" s="27"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="B9" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="D9" s="27">
+        <v>7.0</v>
+      </c>
+      <c r="E9" s="27">
+        <v>2.0</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
+      <c r="C10" s="27" t="s">
+        <v>239</v>
+      </c>
+      <c r="D10" s="27">
+        <v>7.0</v>
+      </c>
+      <c r="E10" s="27">
+        <v>2.0</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
+      <c r="C11" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="D11" s="27">
+        <v>5.0</v>
+      </c>
+      <c r="E11" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
+      <c r="C12" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="D12" s="27">
+        <v>6.0</v>
+      </c>
+      <c r="E12" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="B13" s="24"/>
@@ -10879,6 +10977,11 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B9:B12"/>
+  </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Limpia el documento de modelado, mejora legibilidad y corrige inconsistencias de información, también actualiza el HTML
</commit_message>
<xml_diff>
--- a/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -8372,7 +8372,7 @@
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="20" t="s">
         <v>218</v>
       </c>
       <c r="D6" s="20">
@@ -9702,8 +9702,8 @@
       <c r="D7" s="20">
         <v>10.0</v>
       </c>
-      <c r="E7" s="20">
-        <v>2.0</v>
+      <c r="E7" s="22">
+        <v>1.0</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>230</v>

</xml_diff>